<commit_message>
Trim test ideas list to ID, Type and Test Idea
Drop the Source and Notes columns and the folder README.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ECSE_Test_Ideas_002/Test_Ideas_List.xlsx
+++ b/ECSE_Test_Ideas_002/Test_Ideas_List.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Test Ideas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Ideas'!$A$1:$E$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Ideas'!$A$1:$C$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,14 +452,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="96" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -478,16 +476,6 @@
           <t>Test Idea</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Source (Product Variable Map)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
     </row>
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -505,16 +493,6 @@
           <t>Whether the wrapper seals correctly for all 7 chocolate configurations (truffle, praline, bar, turtle, bon bon, filled, traditional) across all 3 sizes.</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Inputs &gt; Chocolates &gt; Configuration, Size</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>21 combinations. Sample one size per configuration first, widen only where a seal fails.</t>
-        </is>
-      </c>
     </row>
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -532,16 +510,6 @@
           <t>Whether an entered manifest drives correct box layout for every box type (rectangular, circular, heart, OEM custom, bag), size, and layer count.</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Inputs &gt; Manifest; Inputs &gt; Empty Boxes &gt; Type, Size, Configuration</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Covers the manifest-to-layout mapping, not the wrapping itself. OEM custom is the likely weak point.</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -559,16 +527,6 @@
           <t>What the machine does when wrapping paper runs out mid-run: stop, reject, or keep boxing unwrapped chocolates while reporting a normal run.</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Inputs &gt; Paper &gt; None; Users &gt; Loader &gt; Chocolate Wrapping Paper</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Silent under-reporting is the costly outcome. Check the prod run report as well as the belt.</t>
-        </is>
-      </c>
     </row>
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -586,16 +544,6 @@
           <t>Whether out-of-spec chocolates (too light, too heavy, jelly, hollow) divert to the reject output instead of jamming or crushing inside the wrapper.</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Inputs &gt; Chocolates &gt; Weight, Viscosity; Outputs &gt; Rejected Chocolates</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Hollow and jelly are the physical extremes. Jam recovery time is worth recording.</t>
-        </is>
-      </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -613,16 +561,6 @@
           <t>Whether wrap quality and reject rate hold as conveyor speed steps slow to very fast under a dense, randomly distributed input stream.</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Inputs &gt; Input Stream &gt; Conveyor Speed, Frequency, Distribution</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Performance. Random distribution at very fast is the stress corner. Measure reject rate per speed.</t>
-        </is>
-      </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -640,16 +578,6 @@
           <t>Whether a peanut batch is fully purged at changeover so no trace reaches the next peanut-free run, and whether the inspector can prove it.</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Users &gt; Health Inspector &gt; Peanuts, Contamination, Ingredients match labels</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>Safety and compliance. Evidence trail matters as much as the physical purge.</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -667,16 +595,6 @@
           <t>Loader replenishing paper and ribbon in all three states (operating, idle, powered down): whether each is safe, permitted, and logged to stock.</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Users &gt; Loader &gt; Chocolate Wrapping Paper (operating / idle / powered down), Ribbons</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>The map calls out all three states explicitly, so all three are in scope.</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -694,16 +612,6 @@
           <t>Whether an auditor can reconcile prod run, daily, and monthly reports into matching totals after an operator stops and restarts mid-batch.</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Users &gt; Auditor &gt; Batch, Daily, Monthly reports; Users &gt; Operator &gt; Starts, Stops</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>A split batch is where report totals most plausibly drift apart.</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -721,16 +629,6 @@
           <t>Feeding an already-wrapped chocolate back onto the belt: does the machine double-wrap it, reject it, or mis-count it as new production?</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Inputs &gt; Input Stream; Outputs &gt; Wrapped box of chocolates</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Adversarial input the design likely never considered. Cheap to try, high information.</t>
-        </is>
-      </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -748,19 +646,9 @@
           <t>Entering a manifest whose layout cannot physically fit the loaded box (24 large turtles in a small heart box): is it caught before stock is consumed?</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Inputs &gt; Manifest; Inputs &gt; Empty Boxes &gt; Size; Inputs &gt; Chocolates &gt; Size</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>Tests validation timing. Detection after the run has started still wastes chocolate.</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E11"/>
+  <autoFilter ref="A1:C11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Renumber test ideas as TID001 through TID010
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ECSE_Test_Ideas_002/Test_Ideas_List.xlsx
+++ b/ECSE_Test_Ideas_002/Test_Ideas_List.xlsx
@@ -480,7 +480,7 @@
     <row r="2" ht="46" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TI-01</t>
+          <t>TID001</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -497,7 +497,7 @@
     <row r="3" ht="46" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TI-02</t>
+          <t>TID002</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TI-03</t>
+          <t>TID003</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -531,7 +531,7 @@
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TI-04</t>
+          <t>TID004</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -548,7 +548,7 @@
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>TI-05</t>
+          <t>TID005</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -565,7 +565,7 @@
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TI-06</t>
+          <t>TID006</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -582,7 +582,7 @@
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TI-07</t>
+          <t>TID007</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TI-08</t>
+          <t>TID008</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -616,7 +616,7 @@
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TI-09</t>
+          <t>TID009</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -633,7 +633,7 @@
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TI-10</t>
+          <t>TID010</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Rewrite test ideas without parenthetical lists
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ECSE_Test_Ideas_002/Test_Ideas_List.xlsx
+++ b/ECSE_Test_Ideas_002/Test_Ideas_List.xlsx
@@ -455,7 +455,7 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="96" customWidth="1" min="3" max="3"/>
   </cols>
@@ -477,7 +477,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="46" customHeight="1">
+    <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>TID001</t>
@@ -490,11 +490,11 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Whether the wrapper seals correctly for all 7 chocolate configurations (truffle, praline, bar, turtle, bon bon, filled, traditional) across all 3 sizes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="46" customHeight="1">
+          <t>Whether the wrapper produces a sealed, correctly oriented wrap for every chocolate configuration at every size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>TID002</t>
@@ -507,11 +507,11 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Whether an entered manifest drives correct box layout for every box type (rectangular, circular, heart, OEM custom, bag), size, and layer count.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="46" customHeight="1">
+          <t>Whether an entered manifest drives the correct box layout for every box type, size and layer count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>TID003</t>
@@ -524,11 +524,11 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>What the machine does when wrapping paper runs out mid-run: stop, reject, or keep boxing unwrapped chocolates while reporting a normal run.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="46" customHeight="1">
+          <t>What the machine does when wrapping paper runs out mid-run, and whether the run report still reads as normal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>TID004</t>
@@ -541,11 +541,11 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Whether out-of-spec chocolates (too light, too heavy, jelly, hollow) divert to the reject output instead of jamming or crushing inside the wrapper.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="46" customHeight="1">
+          <t>Whether out-of-spec chocolates divert to the reject output instead of jamming the wrapper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>TID005</t>
@@ -558,11 +558,11 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Whether wrap quality and reject rate hold as conveyor speed steps slow to very fast under a dense, randomly distributed input stream.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="46" customHeight="1">
+          <t>Whether wrap quality and reject rate hold as conveyor speed rises to its maximum under a dense, randomly distributed stream.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>TID006</t>
@@ -575,11 +575,11 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Whether a peanut batch is fully purged at changeover so no trace reaches the next peanut-free run, and whether the inspector can prove it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="46" customHeight="1">
+          <t>Whether a peanut batch is fully purged at changeover, and whether the health inspector can prove it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>TID007</t>
@@ -592,11 +592,11 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Loader replenishing paper and ribbon in all three states (operating, idle, powered down): whether each is safe, permitted, and logged to stock.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="46" customHeight="1">
+          <t>Whether a loader can replenish paper and ribbon safely while the line is operating, idle and powered down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>TID008</t>
@@ -609,11 +609,11 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Whether an auditor can reconcile prod run, daily, and monthly reports into matching totals after an operator stops and restarts mid-batch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="46" customHeight="1">
+          <t>Whether an auditor can reconcile prod run, daily and monthly reports after an operator stops and restarts mid-batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>TID009</t>
@@ -626,11 +626,11 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Feeding an already-wrapped chocolate back onto the belt: does the machine double-wrap it, reject it, or mis-count it as new production?</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="46" customHeight="1">
+          <t>Whether an already-wrapped chocolate fed back onto the belt is double-wrapped, rejected, or counted as new production.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>TID010</t>
@@ -643,7 +643,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Entering a manifest whose layout cannot physically fit the loaded box (24 large turtles in a small heart box): is it caught before stock is consumed?</t>
+          <t>Whether a manifest whose layout cannot physically fit the loaded box is caught before stock is consumed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Open each test idea with its type keyword
Confirm, What if, Study and Can, per the exercise convention.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ECSE_Test_Ideas_002/Test_Ideas_List.xlsx
+++ b/ECSE_Test_Ideas_002/Test_Ideas_List.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Whether the wrapper produces a sealed, correctly oriented wrap for every chocolate configuration at every size.</t>
+          <t>Confirm the wrapper produces a sealed, correctly oriented wrap for every chocolate configuration at every size.</t>
         </is>
       </c>
     </row>
@@ -507,7 +507,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Whether an operator's manifest produces the correct box layout for every box type, size and layer count.</t>
+          <t>Confirm an operator's manifest produces the correct box layout for every box type, size and layer count.</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>What the machine does when wrapping paper runs out mid-run, and whether the run report still reads as normal.</t>
+          <t>What if wrapping paper runs out mid-run, does the machine stop or keep boxing unwrapped chocolates and report a normal run?</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Whether out-of-spec chocolates divert to the reject output instead of jamming the wrapper.</t>
+          <t>What if an out-of-spec chocolate reaches the wrapper, does it divert to the reject output or jam the machine?</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Whether wrap quality and reject rate hold as conveyor speed rises to its maximum under a dense, randomly distributed stream.</t>
+          <t>Study how wrap quality and reject rate hold as conveyor speed rises to its maximum under a dense, randomly distributed stream.</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Whether a peanut batch is fully purged at changeover, and whether the health inspector can prove it.</t>
+          <t>Study whether a peanut batch is fully purged at changeover, and whether the health inspector can prove it.</t>
         </is>
       </c>
     </row>
@@ -592,7 +592,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Whether a loader can replenish paper and ribbon safely while the line is operating, idle and powered down.</t>
+          <t>Can a loader replenish paper and ribbon safely while the line is operating, idle and powered down?</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Whether an auditor can reconcile prod run, daily and monthly reports after an operator stops and restarts mid-batch.</t>
+          <t>Can an auditor reconcile prod run, daily and monthly reports after an operator stops and restarts mid-batch?</t>
         </is>
       </c>
     </row>

</xml_diff>